<commit_message>
Fixed CS1022 syntax error in FavoritesService, verified features, and updated issue log spreadsheet
</commit_message>
<xml_diff>
--- a/CountryExplorer/docs/CountryExplorer_Issue_Tracking_Log.xlsx
+++ b/CountryExplorer/docs/CountryExplorer_Issue_Tracking_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\CountryExplorer\CountryExplorer\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D25F04D-D032-4D0B-BABD-32AA4635DBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AAE35F-1E8D-4200-B749-A37B8AE1678B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8244" yWindow="252" windowWidth="14892" windowHeight="11592" xr2:uid="{176F191C-7A5E-4236-BFA1-769CBBA7F852}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>Issue ID</t>
   </si>
@@ -159,6 +159,18 @@
   </si>
   <si>
     <t>Issues Tracking  Table</t>
+  </si>
+  <si>
+    <t>C# Compiler</t>
+  </si>
+  <si>
+    <t>CS1022 error: Type or namespace definition, or end-of-file expected in FavoritesService.cs.</t>
+  </si>
+  <si>
+    <t>Redundant trailing closing curly brace at line 39 of FavoritesService.cs.</t>
+  </si>
+  <si>
+    <t>Deleted extra closing brace at the bottom of the file.</t>
   </si>
 </sst>
 </file>
@@ -829,9 +841,27 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">

</xml_diff>